<commit_message>
chore(assets): update CCS Field labels and filters - Final - PRG - 1 OCT 2026 workbook
Adds the latest local copy of the workbook (record field labels + search filters source of truth).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KSqz6M9upeLSHEDP6tycMx
</commit_message>
<xml_diff>
--- a/assets/CCS Field labels and filters - Final - PRG - 1 OCT 2026.xlsx
+++ b/assets/CCS Field labels and filters - Final - PRG - 1 OCT 2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30524"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud.sharepoint.com/sites/OPGProjects/Initiatives/Cultural Collections Nexus/09 Cross Collection Search 2026 Delivery/06 Product Design Pod/02 Product Design/02 Working Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{122F7D5F-FD2B-4183-934D-8F2C97C8DA87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{86D50DC6-4D2E-46C6-B2A0-59946159918D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17920" xr2:uid="{7E81937D-8799-4F94-A634-A3C622128AD4}"/>
   </bookViews>
@@ -2727,114 +2727,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Project xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <TaxCatchAll xmlns="247916fd-1a60-495e-a02f-9dbb51413255" xsi:nil="true"/>
-    <PID xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <ProjectStartDate xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <ProjectEndDate xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <Status xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Active</Status>
-    <Function xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">DVC Education - Student and Scholarly Services</Function>
-    <DocumentSetDescription xmlns="http://schemas.microsoft.com/sharepoint/v3">Creating, managing and retrieving assets and their associated metadata and rights/permissions details is a significant endeavour for the University with over 100K assets under various management regimes and between 10,000 to 20,000 high important assets digitised each year (Source: 2021 DAM analysis).  
-Currently each collection is independently and sparsely digitised. This leads to inconsistency in the housing, finding and accessing these assets. This creates a security and compliance risk as well as inefficiencies. We have no way of measuring performance of these assets, systematically managing rights, maximising consistency and re-use.
-In SmartSheet PID254 has been closed and replaced with PID365. </DocumentSetDescription>
-    <LinktoCanvas xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <Members xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Members>
-    <Deliverable xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <LeadTeam xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Digital</LeadTeam>
-    <LinktoCloseReport xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </LinktoCloseReport>
-    <ProjectLead xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
-      <UserInfo>
-        <DisplayName>Shona Barrett</DisplayName>
-        <AccountId>1453</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </ProjectLead>
-    <ToolsUsed xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <LinktoStrategy xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <OtherGroups xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <Pillar xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Digital Transformation</Pillar>
-    <LessonsLearned xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_dlc_DocId xmlns="247916fd-1a60-495e-a02f-9dbb51413255">AMZWAK7HTCT4-1043692212-59917</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="247916fd-1a60-495e-a02f-9dbb51413255">
-      <Url>https://unimelbcloud.sharepoint.com/sites/OPGProjects/_layouts/15/DocIdRedir.aspx?ID=AMZWAK7HTCT4-1043692212-59917</Url>
-      <Description>AMZWAK7HTCT4-1043692212-59917</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100107669A72ECB114D9FF76A8CA171E054" ma:contentTypeVersion="46" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="10f9caf407deae0f3f217c6265eabac5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xmlns:ns3="247916fd-1a60-495e-a02f-9dbb51413255" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2de188e63c5f14f3bb9c9b41488d10c7" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3331,18 +3223,126 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Project xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <TaxCatchAll xmlns="247916fd-1a60-495e-a02f-9dbb51413255" xsi:nil="true"/>
+    <PID xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <ProjectStartDate xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <ProjectEndDate xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <Status xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Active</Status>
+    <Function xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">DVC Education - Student and Scholarly Services</Function>
+    <DocumentSetDescription xmlns="http://schemas.microsoft.com/sharepoint/v3">Creating, managing and retrieving assets and their associated metadata and rights/permissions details is a significant endeavour for the University with over 100K assets under various management regimes and between 10,000 to 20,000 high important assets digitised each year (Source: 2021 DAM analysis).  
+Currently each collection is independently and sparsely digitised. This leads to inconsistency in the housing, finding and accessing these assets. This creates a security and compliance risk as well as inefficiencies. We have no way of measuring performance of these assets, systematically managing rights, maximising consistency and re-use.
+In SmartSheet PID254 has been closed and replaced with PID365. </DocumentSetDescription>
+    <LinktoCanvas xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <Members xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Members>
+    <Deliverable xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <LeadTeam xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Digital</LeadTeam>
+    <LinktoCloseReport xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </LinktoCloseReport>
+    <ProjectLead xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
+      <UserInfo>
+        <DisplayName>Shona Barrett</DisplayName>
+        <AccountId>1453</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </ProjectLead>
+    <ToolsUsed xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <LinktoStrategy xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <OtherGroups xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <Pillar xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Digital Transformation</Pillar>
+    <LessonsLearned xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_dlc_DocId xmlns="247916fd-1a60-495e-a02f-9dbb51413255">AMZWAK7HTCT4-1043692212-59917</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="247916fd-1a60-495e-a02f-9dbb51413255">
+      <Url>https://unimelbcloud.sharepoint.com/sites/OPGProjects/_layouts/15/DocIdRedir.aspx?ID=AMZWAK7HTCT4-1043692212-59917</Url>
+      <Description>AMZWAK7HTCT4-1043692212-59917</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{840A8891-0277-4453-B154-09C236A91E67}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A02A138A-A9A0-4A5C-AD13-5146096A96E8}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F96701C4-2080-4DFE-BE16-91280081C66E}"/>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D53C0081-EA6C-4163-9455-3BD588A09F90}"/>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{840A8891-0277-4453-B154-09C236A91E67}"/>
 </file>
</xml_diff>

<commit_message>
chore(assets): update CCS Field labels and filters - Final - PRG - 1 OCT 2026 workbook (#48)
Adds the latest local copy of the workbook (record field labels + search filters source of truth).


Claude-Session: https://claude.ai/code/session_01KSqz6M9upeLSHEDP6tycMx

Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/CCS Field labels and filters - Final - PRG - 1 OCT 2026.xlsx
+++ b/assets/CCS Field labels and filters - Final - PRG - 1 OCT 2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30524"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud.sharepoint.com/sites/OPGProjects/Initiatives/Cultural Collections Nexus/09 Cross Collection Search 2026 Delivery/06 Product Design Pod/02 Product Design/02 Working Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{122F7D5F-FD2B-4183-934D-8F2C97C8DA87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{86D50DC6-4D2E-46C6-B2A0-59946159918D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17920" xr2:uid="{7E81937D-8799-4F94-A634-A3C622128AD4}"/>
   </bookViews>
@@ -2727,114 +2727,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Project xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <TaxCatchAll xmlns="247916fd-1a60-495e-a02f-9dbb51413255" xsi:nil="true"/>
-    <PID xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <ProjectStartDate xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <ProjectEndDate xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <Status xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Active</Status>
-    <Function xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">DVC Education - Student and Scholarly Services</Function>
-    <DocumentSetDescription xmlns="http://schemas.microsoft.com/sharepoint/v3">Creating, managing and retrieving assets and their associated metadata and rights/permissions details is a significant endeavour for the University with over 100K assets under various management regimes and between 10,000 to 20,000 high important assets digitised each year (Source: 2021 DAM analysis).  
-Currently each collection is independently and sparsely digitised. This leads to inconsistency in the housing, finding and accessing these assets. This creates a security and compliance risk as well as inefficiencies. We have no way of measuring performance of these assets, systematically managing rights, maximising consistency and re-use.
-In SmartSheet PID254 has been closed and replaced with PID365. </DocumentSetDescription>
-    <LinktoCanvas xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <Members xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Members>
-    <Deliverable xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <LeadTeam xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Digital</LeadTeam>
-    <LinktoCloseReport xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </LinktoCloseReport>
-    <ProjectLead xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
-      <UserInfo>
-        <DisplayName>Shona Barrett</DisplayName>
-        <AccountId>1453</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </ProjectLead>
-    <ToolsUsed xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <LinktoStrategy xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <OtherGroups xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <Pillar xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Digital Transformation</Pillar>
-    <LessonsLearned xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_dlc_DocId xmlns="247916fd-1a60-495e-a02f-9dbb51413255">AMZWAK7HTCT4-1043692212-59917</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="247916fd-1a60-495e-a02f-9dbb51413255">
-      <Url>https://unimelbcloud.sharepoint.com/sites/OPGProjects/_layouts/15/DocIdRedir.aspx?ID=AMZWAK7HTCT4-1043692212-59917</Url>
-      <Description>AMZWAK7HTCT4-1043692212-59917</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100107669A72ECB114D9FF76A8CA171E054" ma:contentTypeVersion="46" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="10f9caf407deae0f3f217c6265eabac5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xmlns:ns3="247916fd-1a60-495e-a02f-9dbb51413255" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2de188e63c5f14f3bb9c9b41488d10c7" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3331,18 +3223,126 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Project xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <TaxCatchAll xmlns="247916fd-1a60-495e-a02f-9dbb51413255" xsi:nil="true"/>
+    <PID xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <ProjectStartDate xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <ProjectEndDate xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <Status xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Active</Status>
+    <Function xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">DVC Education - Student and Scholarly Services</Function>
+    <DocumentSetDescription xmlns="http://schemas.microsoft.com/sharepoint/v3">Creating, managing and retrieving assets and their associated metadata and rights/permissions details is a significant endeavour for the University with over 100K assets under various management regimes and between 10,000 to 20,000 high important assets digitised each year (Source: 2021 DAM analysis).  
+Currently each collection is independently and sparsely digitised. This leads to inconsistency in the housing, finding and accessing these assets. This creates a security and compliance risk as well as inefficiencies. We have no way of measuring performance of these assets, systematically managing rights, maximising consistency and re-use.
+In SmartSheet PID254 has been closed and replaced with PID365. </DocumentSetDescription>
+    <LinktoCanvas xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <Members xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Members>
+    <Deliverable xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <LeadTeam xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Digital</LeadTeam>
+    <LinktoCloseReport xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </LinktoCloseReport>
+    <ProjectLead xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
+      <UserInfo>
+        <DisplayName>Shona Barrett</DisplayName>
+        <AccountId>1453</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </ProjectLead>
+    <ToolsUsed xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <LinktoStrategy xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <OtherGroups xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <Pillar xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Digital Transformation</Pillar>
+    <LessonsLearned xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_dlc_DocId xmlns="247916fd-1a60-495e-a02f-9dbb51413255">AMZWAK7HTCT4-1043692212-59917</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="247916fd-1a60-495e-a02f-9dbb51413255">
+      <Url>https://unimelbcloud.sharepoint.com/sites/OPGProjects/_layouts/15/DocIdRedir.aspx?ID=AMZWAK7HTCT4-1043692212-59917</Url>
+      <Description>AMZWAK7HTCT4-1043692212-59917</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{840A8891-0277-4453-B154-09C236A91E67}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A02A138A-A9A0-4A5C-AD13-5146096A96E8}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F96701C4-2080-4DFE-BE16-91280081C66E}"/>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D53C0081-EA6C-4163-9455-3BD588A09F90}"/>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{840A8891-0277-4453-B154-09C236A91E67}"/>
 </file>
</xml_diff>

<commit_message>
docs(data): update CCS Field labels and filters spreadsheet (1 Oct 2026); Creator role confirmed as a filter by the data team
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015yontbZMiCaUG2Z46hhMi6
</commit_message>
<xml_diff>
--- a/assets/CCS Field labels and filters - Final - PRG - 1 OCT 2026.xlsx
+++ b/assets/CCS Field labels and filters - Final - PRG - 1 OCT 2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30601"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud.sharepoint.com/sites/OPGProjects/Initiatives/Cultural Collections Nexus/09 Cross Collection Search 2026 Delivery/06 Product Design Pod/02 Product Design/02 Working Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{86D50DC6-4D2E-46C6-B2A0-59946159918D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8424F7F3-85B4-4C1F-ADF4-4C6AAF36B867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17920" xr2:uid="{7E81937D-8799-4F94-A634-A3C622128AD4}"/>
   </bookViews>
@@ -2727,6 +2727,114 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Project xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <TaxCatchAll xmlns="247916fd-1a60-495e-a02f-9dbb51413255" xsi:nil="true"/>
+    <PID xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <ProjectStartDate xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <ProjectEndDate xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <Status xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Active</Status>
+    <Function xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">DVC Education - Student and Scholarly Services</Function>
+    <DocumentSetDescription xmlns="http://schemas.microsoft.com/sharepoint/v3">Creating, managing and retrieving assets and their associated metadata and rights/permissions details is a significant endeavour for the University with over 100K assets under various management regimes and between 10,000 to 20,000 high important assets digitised each year (Source: 2021 DAM analysis).  
+Currently each collection is independently and sparsely digitised. This leads to inconsistency in the housing, finding and accessing these assets. This creates a security and compliance risk as well as inefficiencies. We have no way of measuring performance of these assets, systematically managing rights, maximising consistency and re-use.
+In SmartSheet PID254 has been closed and replaced with PID365. </DocumentSetDescription>
+    <LinktoCanvas xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <Members xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Members>
+    <Deliverable xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <LeadTeam xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Digital</LeadTeam>
+    <LinktoCloseReport xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </LinktoCloseReport>
+    <ProjectLead xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
+      <UserInfo>
+        <DisplayName>Shona Barrett</DisplayName>
+        <AccountId>1453</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </ProjectLead>
+    <ToolsUsed xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <LinktoStrategy xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <OtherGroups xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <Pillar xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Digital Transformation</Pillar>
+    <LessonsLearned xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_dlc_DocId xmlns="247916fd-1a60-495e-a02f-9dbb51413255">AMZWAK7HTCT4-1043692212-59917</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="247916fd-1a60-495e-a02f-9dbb51413255">
+      <Url>https://unimelbcloud.sharepoint.com/sites/OPGProjects/_layouts/15/DocIdRedir.aspx?ID=AMZWAK7HTCT4-1043692212-59917</Url>
+      <Description>AMZWAK7HTCT4-1043692212-59917</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100107669A72ECB114D9FF76A8CA171E054" ma:contentTypeVersion="46" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="10f9caf407deae0f3f217c6265eabac5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xmlns:ns3="247916fd-1a60-495e-a02f-9dbb51413255" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2de188e63c5f14f3bb9c9b41488d10c7" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3223,126 +3331,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Project xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <TaxCatchAll xmlns="247916fd-1a60-495e-a02f-9dbb51413255" xsi:nil="true"/>
-    <PID xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <ProjectStartDate xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <ProjectEndDate xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <Status xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Active</Status>
-    <Function xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">DVC Education - Student and Scholarly Services</Function>
-    <DocumentSetDescription xmlns="http://schemas.microsoft.com/sharepoint/v3">Creating, managing and retrieving assets and their associated metadata and rights/permissions details is a significant endeavour for the University with over 100K assets under various management regimes and between 10,000 to 20,000 high important assets digitised each year (Source: 2021 DAM analysis).  
-Currently each collection is independently and sparsely digitised. This leads to inconsistency in the housing, finding and accessing these assets. This creates a security and compliance risk as well as inefficiencies. We have no way of measuring performance of these assets, systematically managing rights, maximising consistency and re-use.
-In SmartSheet PID254 has been closed and replaced with PID365. </DocumentSetDescription>
-    <LinktoCanvas xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <Members xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Members>
-    <Deliverable xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <LeadTeam xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Digital</LeadTeam>
-    <LinktoCloseReport xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </LinktoCloseReport>
-    <ProjectLead xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
-      <UserInfo>
-        <DisplayName>Shona Barrett</DisplayName>
-        <AccountId>1453</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </ProjectLead>
-    <ToolsUsed xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <LinktoStrategy xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <OtherGroups xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <Pillar xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Digital Transformation</Pillar>
-    <LessonsLearned xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_dlc_DocId xmlns="247916fd-1a60-495e-a02f-9dbb51413255">AMZWAK7HTCT4-1043692212-59917</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="247916fd-1a60-495e-a02f-9dbb51413255">
-      <Url>https://unimelbcloud.sharepoint.com/sites/OPGProjects/_layouts/15/DocIdRedir.aspx?ID=AMZWAK7HTCT4-1043692212-59917</Url>
-      <Description>AMZWAK7HTCT4-1043692212-59917</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{840A8891-0277-4453-B154-09C236A91E67}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A02A138A-A9A0-4A5C-AD13-5146096A96E8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A02A138A-A9A0-4A5C-AD13-5146096A96E8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F96701C4-2080-4DFE-BE16-91280081C66E}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F96701C4-2080-4DFE-BE16-91280081C66E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D53C0081-EA6C-4163-9455-3BD588A09F90}"/>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D53C0081-EA6C-4163-9455-3BD588A09F90}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{840A8891-0277-4453-B154-09C236A91E67}"/>
 </file>
</xml_diff>

<commit_message>
feat(filters): Creator role filter (#114)
* feat(filters): Creator role filter in the Filters modal (Creator group)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015yontbZMiCaUG2Z46hhMi6

* docs(data): update CCS Field labels and filters spreadsheet (1 Oct 2026); Creator role confirmed as a filter by the data team

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015yontbZMiCaUG2Z46hhMi6

---------

Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/CCS Field labels and filters - Final - PRG - 1 OCT 2026.xlsx
+++ b/assets/CCS Field labels and filters - Final - PRG - 1 OCT 2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30601"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud.sharepoint.com/sites/OPGProjects/Initiatives/Cultural Collections Nexus/09 Cross Collection Search 2026 Delivery/06 Product Design Pod/02 Product Design/02 Working Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{86D50DC6-4D2E-46C6-B2A0-59946159918D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8424F7F3-85B4-4C1F-ADF4-4C6AAF36B867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17920" xr2:uid="{7E81937D-8799-4F94-A634-A3C622128AD4}"/>
   </bookViews>
@@ -2727,6 +2727,114 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Project xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <TaxCatchAll xmlns="247916fd-1a60-495e-a02f-9dbb51413255" xsi:nil="true"/>
+    <PID xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <ProjectStartDate xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <ProjectEndDate xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <Status xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Active</Status>
+    <Function xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">DVC Education - Student and Scholarly Services</Function>
+    <DocumentSetDescription xmlns="http://schemas.microsoft.com/sharepoint/v3">Creating, managing and retrieving assets and their associated metadata and rights/permissions details is a significant endeavour for the University with over 100K assets under various management regimes and between 10,000 to 20,000 high important assets digitised each year (Source: 2021 DAM analysis).  
+Currently each collection is independently and sparsely digitised. This leads to inconsistency in the housing, finding and accessing these assets. This creates a security and compliance risk as well as inefficiencies. We have no way of measuring performance of these assets, systematically managing rights, maximising consistency and re-use.
+In SmartSheet PID254 has been closed and replaced with PID365. </DocumentSetDescription>
+    <LinktoCanvas xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <Members xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Members>
+    <Deliverable xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <LeadTeam xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Digital</LeadTeam>
+    <LinktoCloseReport xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </LinktoCloseReport>
+    <ProjectLead xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
+      <UserInfo>
+        <DisplayName>Shona Barrett</DisplayName>
+        <AccountId>1453</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </ProjectLead>
+    <ToolsUsed xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <LinktoStrategy xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <OtherGroups xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <Pillar xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Digital Transformation</Pillar>
+    <LessonsLearned xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_dlc_DocId xmlns="247916fd-1a60-495e-a02f-9dbb51413255">AMZWAK7HTCT4-1043692212-59917</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="247916fd-1a60-495e-a02f-9dbb51413255">
+      <Url>https://unimelbcloud.sharepoint.com/sites/OPGProjects/_layouts/15/DocIdRedir.aspx?ID=AMZWAK7HTCT4-1043692212-59917</Url>
+      <Description>AMZWAK7HTCT4-1043692212-59917</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100107669A72ECB114D9FF76A8CA171E054" ma:contentTypeVersion="46" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="10f9caf407deae0f3f217c6265eabac5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xmlns:ns3="247916fd-1a60-495e-a02f-9dbb51413255" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2de188e63c5f14f3bb9c9b41488d10c7" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3223,126 +3331,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Project xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <TaxCatchAll xmlns="247916fd-1a60-495e-a02f-9dbb51413255" xsi:nil="true"/>
-    <PID xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <ProjectStartDate xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <ProjectEndDate xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <Status xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Active</Status>
-    <Function xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">DVC Education - Student and Scholarly Services</Function>
-    <DocumentSetDescription xmlns="http://schemas.microsoft.com/sharepoint/v3">Creating, managing and retrieving assets and their associated metadata and rights/permissions details is a significant endeavour for the University with over 100K assets under various management regimes and between 10,000 to 20,000 high important assets digitised each year (Source: 2021 DAM analysis).  
-Currently each collection is independently and sparsely digitised. This leads to inconsistency in the housing, finding and accessing these assets. This creates a security and compliance risk as well as inefficiencies. We have no way of measuring performance of these assets, systematically managing rights, maximising consistency and re-use.
-In SmartSheet PID254 has been closed and replaced with PID365. </DocumentSetDescription>
-    <LinktoCanvas xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <Members xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Members>
-    <Deliverable xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <LeadTeam xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Digital</LeadTeam>
-    <LinktoCloseReport xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </LinktoCloseReport>
-    <ProjectLead xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
-      <UserInfo>
-        <DisplayName>Shona Barrett</DisplayName>
-        <AccountId>1453</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </ProjectLead>
-    <ToolsUsed xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <LinktoStrategy xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <OtherGroups xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <Pillar xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">Digital Transformation</Pillar>
-    <LessonsLearned xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c1ec1a7-62a1-4012-8155-c336c8cfdc56">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_dlc_DocId xmlns="247916fd-1a60-495e-a02f-9dbb51413255">AMZWAK7HTCT4-1043692212-59917</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="247916fd-1a60-495e-a02f-9dbb51413255">
-      <Url>https://unimelbcloud.sharepoint.com/sites/OPGProjects/_layouts/15/DocIdRedir.aspx?ID=AMZWAK7HTCT4-1043692212-59917</Url>
-      <Description>AMZWAK7HTCT4-1043692212-59917</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{840A8891-0277-4453-B154-09C236A91E67}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A02A138A-A9A0-4A5C-AD13-5146096A96E8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A02A138A-A9A0-4A5C-AD13-5146096A96E8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F96701C4-2080-4DFE-BE16-91280081C66E}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F96701C4-2080-4DFE-BE16-91280081C66E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D53C0081-EA6C-4163-9455-3BD588A09F90}"/>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D53C0081-EA6C-4163-9455-3BD588A09F90}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{840A8891-0277-4453-B154-09C236A91E67}"/>
 </file>
</xml_diff>